<commit_message>
Drop down is working now fully
</commit_message>
<xml_diff>
--- a/CSE_350_Project_Plan.xlsx
+++ b/CSE_350_Project_Plan.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30601"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a19e270734871b32/6th Term/CSE_350_Intro_to_Software/CSE-350-Group-Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="38" documentId="8_{67ACDB67-83B4-4480-A3DD-8A20E909488F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E84DBC11-5BB7-4B81-AC26-CC0908B0A0C3}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="8_{67ACDB67-83B4-4480-A3DD-8A20E909488F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94A79175-D5F4-47B9-9CF4-699CE1414EE9}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -178,12 +178,48 @@
     <t>Medium</t>
   </si>
   <si>
+    <t>Look into the database set up</t>
+  </si>
+  <si>
+    <t>Start drawing out what we want the UI to look like</t>
+  </si>
+  <si>
+    <t>Help with the background knowledge about weather and database</t>
+  </si>
+  <si>
     <t>Finish up the frame of the website</t>
   </si>
   <si>
+    <t>Finish up putting in the database</t>
+  </si>
+  <si>
+    <t>Finish up with UI design</t>
+  </si>
+  <si>
+    <t>Finish with dataset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wrap up anything that wasn't finished and start back-end </t>
+  </si>
+  <si>
+    <t>Start doing the back-end stuff</t>
+  </si>
+  <si>
+    <t>Start putting the UI design into the program</t>
+  </si>
+  <si>
+    <t>Start doing back-end stuff</t>
+  </si>
+  <si>
     <t>Help finish up applying the UI</t>
   </si>
   <si>
+    <t>Finish back-end stuff</t>
+  </si>
+  <si>
+    <t>Finish applying the UI</t>
+  </si>
+  <si>
     <t>Start testing the website</t>
   </si>
   <si>
@@ -196,9 +232,21 @@
     <t>Start putting all of our written things together</t>
   </si>
   <si>
+    <t>Compile writing</t>
+  </si>
+  <si>
     <t>Review written report and turn it in</t>
   </si>
   <si>
+    <t xml:space="preserve">Review written report </t>
+  </si>
+  <si>
+    <t>Review written report</t>
+  </si>
+  <si>
+    <t>Revire written report</t>
+  </si>
+  <si>
     <t>Sprint Tracker — 10 Weeks</t>
   </si>
   <si>
@@ -232,9 +280,6 @@
     <t>Start applying the UI that we decided on and finish the back-end</t>
   </si>
   <si>
-    <t>Finish applying the UI</t>
-  </si>
-  <si>
     <t>Start the testing phase</t>
   </si>
   <si>
@@ -386,51 +431,6 @@
   </si>
   <si>
     <t>Closed</t>
-  </si>
-  <si>
-    <t>Look into the database set up</t>
-  </si>
-  <si>
-    <t>Start drawing out what we want the UI to look like</t>
-  </si>
-  <si>
-    <t>Help with the background knowledge about weather and database</t>
-  </si>
-  <si>
-    <t>Finish up putting in the database</t>
-  </si>
-  <si>
-    <t>Finish up with UI design</t>
-  </si>
-  <si>
-    <t>Finish with dataset</t>
-  </si>
-  <si>
-    <t>Start putting the UI design into the program</t>
-  </si>
-  <si>
-    <t>Start doing the back-end stuff</t>
-  </si>
-  <si>
-    <t>Start doing back-end stuff</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wrap up anything that wasn't finished and start back-end </t>
-  </si>
-  <si>
-    <t>Finish back-end stuff</t>
-  </si>
-  <si>
-    <t>Compile writing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Review written report </t>
-  </si>
-  <si>
-    <t>Review written report</t>
-  </si>
-  <si>
-    <t>Revire written report</t>
   </si>
 </sst>
 </file>
@@ -440,7 +440,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0&quot;%&quot;"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -527,7 +527,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -557,16 +557,17 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -887,7 +888,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>36</c:v>
+                  <c:v>35</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -896,7 +897,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1591,83 +1592,91 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J33"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="10" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="27.95" customHeight="1">
+      <c r="A1" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="11"/>
       <c r="B3" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="12"/>
+      <c r="C3" s="15"/>
       <c r="D3" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="12"/>
+      <c r="E3" s="15"/>
       <c r="F3" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="12"/>
+      <c r="G3" s="15"/>
       <c r="H3" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="12"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="I3" s="15"/>
+      <c r="J3" s="11"/>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="11"/>
       <c r="B4" s="14">
         <f>COUNTA('Agile Plan'!$B$4:$B$44)</f>
         <v>41</v>
       </c>
-      <c r="C4" s="12"/>
+      <c r="C4" s="15"/>
       <c r="D4" s="14">
         <f>COUNTIF('Agile Plan'!$F$4:$F$44,"Done")</f>
-        <v>5</v>
-      </c>
-      <c r="E4" s="12"/>
+        <v>6</v>
+      </c>
+      <c r="E4" s="15"/>
       <c r="F4" s="14">
         <f>COUNTIF('Agile Plan'!$F$4:$F$44,"In Progress")</f>
         <v>0</v>
       </c>
-      <c r="G4" s="12"/>
+      <c r="G4" s="15"/>
       <c r="H4" s="14">
         <f>COUNTIF('Agile Plan'!$F$4:$F$44,"Blocked")</f>
         <v>0</v>
       </c>
-      <c r="I4" s="12"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B5" s="12"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-    </row>
-    <row r="7" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="I4" s="15"/>
+      <c r="J4" s="11"/>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="11"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="11"/>
+    </row>
+    <row r="7" spans="1:10" ht="23.45">
+      <c r="A7" s="11"/>
       <c r="B7" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="2">
         <f>IF(COUNTA('Agile Plan'!$B$4:$B$44)=0,0,COUNTIF('Agile Plan'!$F$4:$F$44,"Done")/COUNTA('Agile Plan'!$B$4:$B$44))</f>
-        <v>0.12195121951219512</v>
-      </c>
+        <v>0.14634146341463414</v>
+      </c>
+      <c r="D7" s="11"/>
       <c r="E7" s="3" t="s">
         <v>6</v>
       </c>
@@ -1675,6 +1684,7 @@
         <f>COUNTIF('Risks &amp; Issues'!$I$4:$I$23,"Open")</f>
         <v>20</v>
       </c>
+      <c r="G7" s="11"/>
       <c r="H7" s="3" t="s">
         <v>7</v>
       </c>
@@ -1682,8 +1692,9 @@
         <f>COUNTIF('Risks &amp; Issues'!$E$4:$E$23,"High")</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J7" s="11"/>
+    </row>
+    <row r="9" spans="1:10" ht="30" customHeight="1">
       <c r="A9" s="5" t="s">
         <v>8</v>
       </c>
@@ -1696,8 +1707,14 @@
       <c r="D9" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="11"/>
+    </row>
+    <row r="10" spans="1:10">
       <c r="A10" s="3" t="s">
         <v>12</v>
       </c>
@@ -1707,14 +1724,20 @@
       </c>
       <c r="C10" s="3">
         <f>COUNTIFS('Agile Plan'!$D$4:$D$44,A10,'Agile Plan'!$F$4:$F$44,"Done")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D10" s="6">
         <f>IF(B10=0,0,C10/B10)</f>
-        <v>0.18181818181818182</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+        <v>0.27272727272727271</v>
+      </c>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
+      <c r="J10" s="11"/>
+    </row>
+    <row r="11" spans="1:10">
       <c r="A11" s="3" t="s">
         <v>13</v>
       </c>
@@ -1730,8 +1753,14 @@
         <f>IF(B11=0,0,C11/B11)</f>
         <v>0.1</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="11"/>
+      <c r="J11" s="11"/>
+    </row>
+    <row r="12" spans="1:10">
       <c r="A12" s="3" t="s">
         <v>14</v>
       </c>
@@ -1747,8 +1776,14 @@
         <f>IF(B12=0,0,C12/B12)</f>
         <v>0.1</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="11"/>
+      <c r="J12" s="11"/>
+    </row>
+    <row r="13" spans="1:10">
       <c r="A13" s="3" t="s">
         <v>15</v>
       </c>
@@ -1764,8 +1799,14 @@
         <f>IF(B13=0,0,C13/B13)</f>
         <v>0.1</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
+      <c r="J13" s="11"/>
+    </row>
+    <row r="16" spans="1:10" ht="30" customHeight="1">
       <c r="A16" s="5" t="s">
         <v>16</v>
       </c>
@@ -1781,8 +1822,13 @@
       <c r="E16" s="5" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
+      <c r="J16" s="11"/>
+    </row>
+    <row r="17" spans="1:5">
       <c r="A17" s="3">
         <v>1</v>
       </c>
@@ -1803,7 +1849,7 @@
         <v>Not Started</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5">
       <c r="A18" s="3">
         <v>2</v>
       </c>
@@ -1824,7 +1870,7 @@
         <v>Not Started</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5">
       <c r="A19" s="3">
         <v>3</v>
       </c>
@@ -1845,7 +1891,7 @@
         <v>Not Started</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5">
       <c r="A20" s="3">
         <v>4</v>
       </c>
@@ -1866,7 +1912,7 @@
         <v>Not Started</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5">
       <c r="A21" s="3">
         <v>5</v>
       </c>
@@ -1887,7 +1933,7 @@
         <v>Not Started</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5">
       <c r="A22" s="3">
         <v>6</v>
       </c>
@@ -1908,7 +1954,7 @@
         <v>Not Started</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5">
       <c r="A23" s="3">
         <v>7</v>
       </c>
@@ -1929,7 +1975,7 @@
         <v>Not Started</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5">
       <c r="A24" s="3">
         <v>8</v>
       </c>
@@ -1950,7 +1996,7 @@
         <v>Not Started</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5">
       <c r="A25" s="3">
         <v>9</v>
       </c>
@@ -1971,7 +2017,7 @@
         <v>Not Started</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5">
       <c r="A26" s="3">
         <v>10</v>
       </c>
@@ -1992,24 +2038,30 @@
         <v>Not Started</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" ht="30" customHeight="1">
       <c r="A29" s="5" t="s">
         <v>20</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="C29" s="11"/>
+      <c r="D29" s="11"/>
+      <c r="E29" s="11"/>
+    </row>
+    <row r="30" spans="1:5">
       <c r="A30" s="3" t="s">
         <v>22</v>
       </c>
       <c r="B30" s="3">
         <f>COUNTIF('Agile Plan'!$F$4:$F$44,A30)</f>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+        <v>35</v>
+      </c>
+      <c r="C30" s="11"/>
+      <c r="D30" s="11"/>
+      <c r="E30" s="11"/>
+    </row>
+    <row r="31" spans="1:5">
       <c r="A31" s="3" t="s">
         <v>3</v>
       </c>
@@ -2017,8 +2069,11 @@
         <f>COUNTIF('Agile Plan'!$F$4:$F$44,A31)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="C31" s="11"/>
+      <c r="D31" s="11"/>
+      <c r="E31" s="11"/>
+    </row>
+    <row r="32" spans="1:5">
       <c r="A32" s="3" t="s">
         <v>4</v>
       </c>
@@ -2026,14 +2081,17 @@
         <f>COUNTIF('Agile Plan'!$F$4:$F$44,A32)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C32" s="11"/>
+      <c r="D32" s="11"/>
+      <c r="E32" s="11"/>
+    </row>
+    <row r="33" spans="1:2">
       <c r="A33" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B33" s="3">
         <f>COUNTIF('Agile Plan'!$F$4:$F$44,A33)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -2057,7 +2115,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:L44"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
@@ -2071,23 +2129,23 @@
     <col min="12" max="12" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:12" ht="27.95" customHeight="1">
+      <c r="A1" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-    </row>
-    <row r="3" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+    </row>
+    <row r="3" spans="1:12" ht="30" customHeight="1">
       <c r="A3" s="5" t="s">
         <v>16</v>
       </c>
@@ -2125,7 +2183,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12">
       <c r="A4" s="7">
         <v>1</v>
       </c>
@@ -2160,7 +2218,7 @@
       </c>
       <c r="L4" s="7"/>
     </row>
-    <row r="5" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" ht="29.1">
       <c r="A5" s="7">
         <v>1</v>
       </c>
@@ -2195,7 +2253,7 @@
       </c>
       <c r="L5" s="7"/>
     </row>
-    <row r="6" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" ht="43.5">
       <c r="A6" s="7">
         <v>1</v>
       </c>
@@ -2224,7 +2282,7 @@
       </c>
       <c r="L6" s="7"/>
     </row>
-    <row r="7" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" ht="29.1">
       <c r="A7" s="7">
         <v>1</v>
       </c>
@@ -2253,7 +2311,7 @@
       </c>
       <c r="L7" s="7"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12">
       <c r="A8" s="7">
         <v>1</v>
       </c>
@@ -2282,7 +2340,7 @@
       </c>
       <c r="L8" s="7"/>
     </row>
-    <row r="9" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" ht="30.75">
       <c r="A9" s="7">
         <v>2</v>
       </c>
@@ -2299,26 +2357,30 @@
         <v>43</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
+        <v>23</v>
+      </c>
+      <c r="G9" s="8">
+        <v>46297</v>
+      </c>
+      <c r="H9" s="8">
+        <v>46298</v>
+      </c>
       <c r="I9" s="7">
         <v>6</v>
       </c>
       <c r="J9" s="7"/>
       <c r="K9" s="9">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="L9" s="7"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12">
       <c r="A10" s="7">
         <v>2</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>114</v>
+        <v>44</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>36</v>
@@ -2342,12 +2404,12 @@
       </c>
       <c r="L10" s="7"/>
     </row>
-    <row r="11" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" ht="29.1">
       <c r="A11" s="7">
         <v>2</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>115</v>
+        <v>45</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>36</v>
@@ -2371,12 +2433,12 @@
       </c>
       <c r="L11" s="7"/>
     </row>
-    <row r="12" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" ht="43.5">
       <c r="A12" s="7">
         <v>2</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>116</v>
+        <v>46</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>36</v>
@@ -2400,12 +2462,12 @@
       </c>
       <c r="L12" s="7"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12">
       <c r="A13" s="7">
         <v>3</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>36</v>
@@ -2429,12 +2491,12 @@
       </c>
       <c r="L13" s="7"/>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12">
       <c r="A14" s="7">
         <v>3</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>117</v>
+        <v>48</v>
       </c>
       <c r="C14" s="7" t="s">
         <v>36</v>
@@ -2458,12 +2520,12 @@
       </c>
       <c r="L14" s="7"/>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12">
       <c r="A15" s="7">
         <v>3</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>118</v>
+        <v>49</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>36</v>
@@ -2487,12 +2549,12 @@
       </c>
       <c r="L15" s="7"/>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12">
       <c r="A16" s="7">
         <v>3</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>119</v>
+        <v>50</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>36</v>
@@ -2516,12 +2578,12 @@
       </c>
       <c r="L16" s="7"/>
     </row>
-    <row r="17" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" ht="29.1">
       <c r="A17" s="7">
         <v>4</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>123</v>
+        <v>51</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>36</v>
@@ -2545,12 +2607,12 @@
       </c>
       <c r="L17" s="7"/>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12">
       <c r="A18" s="7">
         <v>4</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>121</v>
+        <v>52</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>36</v>
@@ -2574,12 +2636,12 @@
       </c>
       <c r="L18" s="7"/>
     </row>
-    <row r="19" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" ht="29.1">
       <c r="A19" s="7">
         <v>4</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>120</v>
+        <v>53</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>36</v>
@@ -2603,12 +2665,12 @@
       </c>
       <c r="L19" s="7"/>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12">
       <c r="A20" s="7">
         <v>4</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>122</v>
+        <v>54</v>
       </c>
       <c r="C20" s="7" t="s">
         <v>36</v>
@@ -2632,12 +2694,12 @@
       </c>
       <c r="L20" s="7"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12">
       <c r="A21" s="7">
         <v>5</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C21" s="7" t="s">
         <v>36</v>
@@ -2661,12 +2723,12 @@
       </c>
       <c r="L21" s="7"/>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12">
       <c r="A22" s="7">
         <v>5</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>124</v>
+        <v>56</v>
       </c>
       <c r="C22" s="7" t="s">
         <v>36</v>
@@ -2690,12 +2752,12 @@
       </c>
       <c r="L22" s="7"/>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12">
       <c r="A23" s="7">
         <v>5</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="C23" s="7" t="s">
         <v>36</v>
@@ -2719,12 +2781,12 @@
       </c>
       <c r="L23" s="7"/>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12">
       <c r="A24" s="7">
         <v>5</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>124</v>
+        <v>56</v>
       </c>
       <c r="C24" s="7" t="s">
         <v>36</v>
@@ -2748,12 +2810,12 @@
       </c>
       <c r="L24" s="7"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12">
       <c r="A25" s="7">
         <v>6</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>36</v>
@@ -2777,12 +2839,12 @@
       </c>
       <c r="L25" s="7"/>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12">
       <c r="A26" s="7">
         <v>6</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="C26" s="7" t="s">
         <v>36</v>
@@ -2806,12 +2868,12 @@
       </c>
       <c r="L26" s="7"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12">
       <c r="A27" s="7">
         <v>6</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="C27" s="7" t="s">
         <v>36</v>
@@ -2835,12 +2897,12 @@
       </c>
       <c r="L27" s="7"/>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12">
       <c r="A28" s="7">
         <v>6</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="C28" s="7" t="s">
         <v>36</v>
@@ -2864,12 +2926,12 @@
       </c>
       <c r="L28" s="7"/>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12">
       <c r="A29" s="7">
         <v>7</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="C29" s="7" t="s">
         <v>36</v>
@@ -2893,12 +2955,12 @@
       </c>
       <c r="L29" s="7"/>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12">
       <c r="A30" s="7">
         <v>7</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="C30" s="7" t="s">
         <v>36</v>
@@ -2922,12 +2984,12 @@
       </c>
       <c r="L30" s="7"/>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12">
       <c r="A31" s="7">
         <v>7</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="C31" s="7" t="s">
         <v>36</v>
@@ -2951,12 +3013,12 @@
       </c>
       <c r="L31" s="7"/>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12">
       <c r="A32" s="7">
         <v>7</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="C32" s="7" t="s">
         <v>36</v>
@@ -2980,12 +3042,12 @@
       </c>
       <c r="L32" s="7"/>
     </row>
-    <row r="33" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" ht="29.1">
       <c r="A33" s="7">
         <v>8</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="C33" s="7" t="s">
         <v>36</v>
@@ -3009,12 +3071,12 @@
       </c>
       <c r="L33" s="7"/>
     </row>
-    <row r="34" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" ht="29.1">
       <c r="A34" s="7">
         <v>8</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="C34" s="7" t="s">
         <v>36</v>
@@ -3038,12 +3100,12 @@
       </c>
       <c r="L34" s="7"/>
     </row>
-    <row r="35" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" ht="29.1">
       <c r="A35" s="7">
         <v>8</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="C35" s="7" t="s">
         <v>36</v>
@@ -3067,12 +3129,12 @@
       </c>
       <c r="L35" s="7"/>
     </row>
-    <row r="36" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" ht="29.1">
       <c r="A36" s="7">
         <v>8</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="C36" s="7" t="s">
         <v>36</v>
@@ -3096,12 +3158,12 @@
       </c>
       <c r="L36" s="7"/>
     </row>
-    <row r="37" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" ht="29.1">
       <c r="A37" s="7">
         <v>9</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="C37" s="7" t="s">
         <v>36</v>
@@ -3125,12 +3187,12 @@
       </c>
       <c r="L37" s="7"/>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12">
       <c r="A38" s="7">
         <v>9</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>125</v>
+        <v>62</v>
       </c>
       <c r="C38" s="7" t="s">
         <v>36</v>
@@ -3154,12 +3216,12 @@
       </c>
       <c r="L38" s="7"/>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12">
       <c r="A39" s="7">
         <v>9</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>125</v>
+        <v>62</v>
       </c>
       <c r="C39" s="7" t="s">
         <v>36</v>
@@ -3183,12 +3245,12 @@
       </c>
       <c r="L39" s="7"/>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:12">
       <c r="A40" s="7">
         <v>9</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>125</v>
+        <v>62</v>
       </c>
       <c r="C40" s="7" t="s">
         <v>36</v>
@@ -3212,12 +3274,12 @@
       </c>
       <c r="L40" s="7"/>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:12">
       <c r="A41" s="7">
         <v>10</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="C41" s="7" t="s">
         <v>36</v>
@@ -3241,12 +3303,12 @@
       </c>
       <c r="L41" s="7"/>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:12">
       <c r="A42" s="7">
         <v>10</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>126</v>
+        <v>64</v>
       </c>
       <c r="C42" s="7" t="s">
         <v>36</v>
@@ -3270,12 +3332,12 @@
       </c>
       <c r="L42" s="7"/>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:12">
       <c r="A43" s="7">
         <v>10</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>127</v>
+        <v>65</v>
       </c>
       <c r="C43" s="7" t="s">
         <v>36</v>
@@ -3299,12 +3361,12 @@
       </c>
       <c r="L43" s="7"/>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:12">
       <c r="A44" s="7">
         <v>10</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>128</v>
+        <v>66</v>
       </c>
       <c r="C44" s="7" t="s">
         <v>36</v>
@@ -3382,7 +3444,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
@@ -3396,39 +3458,39 @@
     <col min="11" max="11" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-    </row>
-    <row r="3" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" ht="27.95" customHeight="1">
+      <c r="A1" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+    </row>
+    <row r="3" spans="1:11" ht="30" customHeight="1">
       <c r="A3" s="5" t="s">
         <v>16</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>17</v>
@@ -3443,15 +3505,15 @@
         <v>19</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
       <c r="A4" s="3">
         <v>1</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
       <c r="C4" s="3">
         <f>SUMIFS('Agile Plan'!$I$4:$I$44,'Agile Plan'!$A$4:$A$44,$A4,'Agile Plan'!$D$4:$D$44,C$3)</f>
@@ -3485,13 +3547,14 @@
         <f t="shared" ref="J4:J13" si="2">IF(I4&gt;=1,"Complete",IF(I4&gt;0,"In Progress","Not Started"))</f>
         <v>Not Started</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K4" s="11"/>
+    </row>
+    <row r="5" spans="1:11" ht="43.5">
       <c r="A5" s="3">
         <v>2</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>59</v>
+        <v>75</v>
       </c>
       <c r="C5" s="3">
         <f>SUMIFS('Agile Plan'!$I$4:$I$44,'Agile Plan'!$A$4:$A$44,$A5,'Agile Plan'!$D$4:$D$44,C$3)</f>
@@ -3525,13 +3588,14 @@
         <f t="shared" si="2"/>
         <v>Not Started</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+      <c r="K5" s="11"/>
+    </row>
+    <row r="6" spans="1:11" ht="29.1">
       <c r="A6" s="3">
         <v>3</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="C6" s="3">
         <f>SUMIFS('Agile Plan'!$I$4:$I$44,'Agile Plan'!$A$4:$A$44,$A6,'Agile Plan'!$D$4:$D$44,C$3)</f>
@@ -3565,13 +3629,14 @@
         <f t="shared" si="2"/>
         <v>Not Started</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+      <c r="K6" s="11"/>
+    </row>
+    <row r="7" spans="1:11" ht="29.1">
       <c r="A7" s="3">
         <v>4</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="C7" s="3">
         <f>SUMIFS('Agile Plan'!$I$4:$I$44,'Agile Plan'!$A$4:$A$44,$A7,'Agile Plan'!$D$4:$D$44,C$3)</f>
@@ -3605,13 +3670,14 @@
         <f t="shared" si="2"/>
         <v>Not Started</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="K7" s="11"/>
+    </row>
+    <row r="8" spans="1:11">
       <c r="A8" s="3">
         <v>5</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="C8" s="3">
         <f>SUMIFS('Agile Plan'!$I$4:$I$44,'Agile Plan'!$A$4:$A$44,$A8,'Agile Plan'!$D$4:$D$44,C$3)</f>
@@ -3645,13 +3711,14 @@
         <f t="shared" si="2"/>
         <v>Not Started</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="K8" s="11"/>
+    </row>
+    <row r="9" spans="1:11">
       <c r="A9" s="3">
         <v>6</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="C9" s="3">
         <f>SUMIFS('Agile Plan'!$I$4:$I$44,'Agile Plan'!$A$4:$A$44,$A9,'Agile Plan'!$D$4:$D$44,C$3)</f>
@@ -3685,13 +3752,14 @@
         <f t="shared" si="2"/>
         <v>Not Started</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+      <c r="K9" s="11"/>
+    </row>
+    <row r="10" spans="1:11" ht="29.1">
       <c r="A10" s="3">
         <v>7</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="C10" s="3">
         <f>SUMIFS('Agile Plan'!$I$4:$I$44,'Agile Plan'!$A$4:$A$44,$A10,'Agile Plan'!$D$4:$D$44,C$3)</f>
@@ -3725,13 +3793,14 @@
         <f t="shared" si="2"/>
         <v>Not Started</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+      <c r="K10" s="11"/>
+    </row>
+    <row r="11" spans="1:11" ht="29.1">
       <c r="A11" s="3">
         <v>8</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="C11" s="3">
         <f>SUMIFS('Agile Plan'!$I$4:$I$44,'Agile Plan'!$A$4:$A$44,$A11,'Agile Plan'!$D$4:$D$44,C$3)</f>
@@ -3765,13 +3834,14 @@
         <f t="shared" si="2"/>
         <v>Not Started</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="K11" s="11"/>
+    </row>
+    <row r="12" spans="1:11">
       <c r="A12" s="3">
         <v>9</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>66</v>
+        <v>81</v>
       </c>
       <c r="C12" s="3">
         <f>SUMIFS('Agile Plan'!$I$4:$I$44,'Agile Plan'!$A$4:$A$44,$A12,'Agile Plan'!$D$4:$D$44,C$3)</f>
@@ -3805,13 +3875,14 @@
         <f t="shared" si="2"/>
         <v>Not Started</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="K12" s="11"/>
+    </row>
+    <row r="13" spans="1:11">
       <c r="A13" s="3">
         <v>10</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>67</v>
+        <v>82</v>
       </c>
       <c r="C13" s="3">
         <f>SUMIFS('Agile Plan'!$I$4:$I$44,'Agile Plan'!$A$4:$A$44,$A13,'Agile Plan'!$D$4:$D$44,C$3)</f>
@@ -3845,6 +3916,7 @@
         <f t="shared" si="2"/>
         <v>Not Started</v>
       </c>
+      <c r="K13" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3858,7 +3930,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:J23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -3872,41 +3944,41 @@
     <col min="10" max="10" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-    </row>
-    <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="27.95" customHeight="1">
+      <c r="A1" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+    </row>
+    <row r="3" spans="1:10" ht="30" customHeight="1">
       <c r="A3" s="5" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>27</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>74</v>
+        <v>89</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>30</v>
@@ -3915,12 +3987,12 @@
         <v>20</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
       <c r="A4" s="7" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="B4" s="8"/>
       <c r="C4" s="7"/>
@@ -3932,13 +4004,13 @@
       <c r="G4" s="7"/>
       <c r="H4" s="8"/>
       <c r="I4" s="7" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="J4" s="7"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10">
       <c r="A5" s="7" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="7"/>
@@ -3950,13 +4022,13 @@
       <c r="G5" s="7"/>
       <c r="H5" s="8"/>
       <c r="I5" s="7" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="J5" s="7"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10">
       <c r="A6" s="7" t="s">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="B6" s="8"/>
       <c r="C6" s="7"/>
@@ -3968,13 +4040,13 @@
       <c r="G6" s="7"/>
       <c r="H6" s="8"/>
       <c r="I6" s="7" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="J6" s="7"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10">
       <c r="A7" s="7" t="s">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="B7" s="8"/>
       <c r="C7" s="7"/>
@@ -3986,13 +4058,13 @@
       <c r="G7" s="7"/>
       <c r="H7" s="8"/>
       <c r="I7" s="7" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="J7" s="7"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10">
       <c r="A8" s="7" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="7"/>
@@ -4004,13 +4076,13 @@
       <c r="G8" s="7"/>
       <c r="H8" s="8"/>
       <c r="I8" s="7" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="J8" s="7"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10">
       <c r="A9" s="7" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="B9" s="8"/>
       <c r="C9" s="7"/>
@@ -4022,13 +4094,13 @@
       <c r="G9" s="7"/>
       <c r="H9" s="8"/>
       <c r="I9" s="7" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="J9" s="7"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10">
       <c r="A10" s="7" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="7"/>
@@ -4040,13 +4112,13 @@
       <c r="G10" s="7"/>
       <c r="H10" s="8"/>
       <c r="I10" s="7" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="J10" s="7"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10">
       <c r="A11" s="7" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="B11" s="8"/>
       <c r="C11" s="7"/>
@@ -4058,13 +4130,13 @@
       <c r="G11" s="7"/>
       <c r="H11" s="8"/>
       <c r="I11" s="7" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="J11" s="7"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10">
       <c r="A12" s="7" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="7"/>
@@ -4076,13 +4148,13 @@
       <c r="G12" s="7"/>
       <c r="H12" s="8"/>
       <c r="I12" s="7" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="J12" s="7"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10">
       <c r="A13" s="7" t="s">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="7"/>
@@ -4094,13 +4166,13 @@
       <c r="G13" s="7"/>
       <c r="H13" s="8"/>
       <c r="I13" s="7" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="J13" s="7"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10">
       <c r="A14" s="7" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="B14" s="8"/>
       <c r="C14" s="7"/>
@@ -4112,13 +4184,13 @@
       <c r="G14" s="7"/>
       <c r="H14" s="8"/>
       <c r="I14" s="7" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="J14" s="7"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10">
       <c r="A15" s="7" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="7"/>
@@ -4130,13 +4202,13 @@
       <c r="G15" s="7"/>
       <c r="H15" s="8"/>
       <c r="I15" s="7" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="J15" s="7"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10">
       <c r="A16" s="7" t="s">
-        <v>89</v>
+        <v>104</v>
       </c>
       <c r="B16" s="8"/>
       <c r="C16" s="7"/>
@@ -4148,13 +4220,13 @@
       <c r="G16" s="7"/>
       <c r="H16" s="8"/>
       <c r="I16" s="7" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="J16" s="7"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10">
       <c r="A17" s="7" t="s">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="7"/>
@@ -4166,13 +4238,13 @@
       <c r="G17" s="7"/>
       <c r="H17" s="8"/>
       <c r="I17" s="7" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="J17" s="7"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10">
       <c r="A18" s="7" t="s">
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="B18" s="8"/>
       <c r="C18" s="7"/>
@@ -4184,13 +4256,13 @@
       <c r="G18" s="7"/>
       <c r="H18" s="8"/>
       <c r="I18" s="7" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="J18" s="7"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10">
       <c r="A19" s="7" t="s">
-        <v>92</v>
+        <v>107</v>
       </c>
       <c r="B19" s="8"/>
       <c r="C19" s="7"/>
@@ -4202,13 +4274,13 @@
       <c r="G19" s="7"/>
       <c r="H19" s="8"/>
       <c r="I19" s="7" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="J19" s="7"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10">
       <c r="A20" s="7" t="s">
-        <v>93</v>
+        <v>108</v>
       </c>
       <c r="B20" s="8"/>
       <c r="C20" s="7"/>
@@ -4220,13 +4292,13 @@
       <c r="G20" s="7"/>
       <c r="H20" s="8"/>
       <c r="I20" s="7" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="J20" s="7"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10">
       <c r="A21" s="7" t="s">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="7"/>
@@ -4238,13 +4310,13 @@
       <c r="G21" s="7"/>
       <c r="H21" s="8"/>
       <c r="I21" s="7" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="J21" s="7"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10">
       <c r="A22" s="7" t="s">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="7"/>
@@ -4256,13 +4328,13 @@
       <c r="G22" s="7"/>
       <c r="H22" s="8"/>
       <c r="I22" s="7" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="J22" s="7"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10">
       <c r="A23" s="7" t="s">
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="7"/>
@@ -4274,7 +4346,7 @@
       <c r="G23" s="7"/>
       <c r="H23" s="8"/>
       <c r="I23" s="7" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="J23" s="7"/>
     </row>
@@ -4322,7 +4394,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
     <col min="2" max="4" width="40" customWidth="1"/>
@@ -4331,41 +4403,41 @@
     <col min="7" max="7" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-    </row>
-    <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="27.95" customHeight="1">
+      <c r="A1" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+    </row>
+    <row r="3" spans="1:7" ht="30" customHeight="1">
       <c r="A3" s="5" t="s">
         <v>16</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
       <c r="A4" s="7">
         <v>1</v>
       </c>
@@ -4378,7 +4450,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7">
       <c r="A5" s="7">
         <v>2</v>
       </c>
@@ -4391,7 +4463,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7">
       <c r="A6" s="7">
         <v>3</v>
       </c>
@@ -4404,7 +4476,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7">
       <c r="A7" s="7">
         <v>4</v>
       </c>
@@ -4417,7 +4489,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7">
       <c r="A8" s="7">
         <v>5</v>
       </c>
@@ -4430,7 +4502,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7">
       <c r="A9" s="7">
         <v>6</v>
       </c>
@@ -4443,7 +4515,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7">
       <c r="A10" s="7">
         <v>7</v>
       </c>
@@ -4456,7 +4528,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7">
       <c r="A11" s="7">
         <v>8</v>
       </c>
@@ -4469,7 +4541,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7">
       <c r="A12" s="7">
         <v>9</v>
       </c>
@@ -4482,7 +4554,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7">
       <c r="A13" s="7">
         <v>10</v>
       </c>
@@ -4528,22 +4600,24 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="6" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" ht="27.95" customHeight="1">
+      <c r="A1" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" s="10" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>20</v>
@@ -4555,13 +4629,13 @@
         <v>26</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4" s="3" t="s">
         <v>12</v>
       </c>
@@ -4575,13 +4649,13 @@
         <v>36</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6">
       <c r="A5" s="3" t="s">
         <v>13</v>
       </c>
@@ -4592,16 +4666,16 @@
         <v>43</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6">
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
@@ -4609,31 +4683,33 @@
         <v>4</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>23</v>
       </c>
+      <c r="C7" s="11"/>
       <c r="D7" s="3" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>113</v>
-      </c>
+        <v>128</v>
+      </c>
+      <c r="F7" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>